<commit_message>
Doc: adiçã de dois requisitos não funcionais
</commit_message>
<xml_diff>
--- a/documentacao/requisitos.xlsx
+++ b/documentacao/requisitos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\Projeto, Oh my dog\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vieira\Desktop\Petsenai\documentacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{901FAA37-A032-4E7F-A6A0-8BF2B2C1EE59}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B24BEC16-77CC-482E-A7E0-3F0E831381FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{9C44EC18-CB13-4539-9BBD-338C7ACFB87E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>REQUISITOS FUNCIONAIS</t>
   </si>
@@ -154,6 +154,18 @@
   <si>
     <t>O SISTEMA DEVE CONTER UMA 
 INTERFACE FACILMENTE INTERATIVA PARA O USUÁRIO ENCONTRAR COM FACILIDADE O QUE BUSCA.</t>
+  </si>
+  <si>
+    <t>RNF_07</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ TER UMA PÁGINA DE LOGIN PARA OS USUÁRIOS FAZEREM O CADASTRO.</t>
+  </si>
+  <si>
+    <t>RNF_08</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE TER UMA PÁGINA PARA O CARRINHO, PARA O USUÁRIO ADICIONAR OU EXCLUIR O QUE FOR SELECIONADO.</t>
   </si>
 </sst>
 </file>
@@ -187,12 +199,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7ADC96"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -230,6 +236,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -295,85 +307,94 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -392,6 +413,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCCFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -704,276 +730,316 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="L1" s="13" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="L1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
     </row>
     <row r="2" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="18"/>
+      <c r="H2" s="7"/>
       <c r="L2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10" t="s">
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="10"/>
+      <c r="S2" s="22"/>
     </row>
     <row r="3" spans="1:19" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="15" t="s">
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="15"/>
+      <c r="H3" s="16"/>
       <c r="L3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="14" t="s">
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="14"/>
+      <c r="S3" s="23"/>
     </row>
     <row r="4" spans="1:19" ht="108" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="16" t="s">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="17"/>
+      <c r="H4" s="18"/>
       <c r="L4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="M4" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="12" t="s">
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="S4" s="12"/>
+      <c r="S4" s="14"/>
     </row>
     <row r="5" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="16" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="17"/>
+      <c r="H5" s="18"/>
       <c r="L5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="M5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="10" t="s">
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="S5" s="10"/>
+      <c r="S5" s="22"/>
     </row>
     <row r="6" spans="1:19" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="16" t="s">
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="17"/>
+      <c r="H6" s="18"/>
       <c r="L6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="M6" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="10" t="s">
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="S6" s="10"/>
+      <c r="S6" s="22"/>
     </row>
     <row r="7" spans="1:19" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="18" t="s">
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="18"/>
+      <c r="H7" s="7"/>
       <c r="L7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="M7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="12" t="s">
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="12"/>
+      <c r="S7" s="14"/>
     </row>
     <row r="8" spans="1:19" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="18" t="s">
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="18"/>
+      <c r="H8" s="7"/>
       <c r="L8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="M8" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="9" t="s">
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="S8" s="9"/>
+      <c r="S8" s="24"/>
     </row>
     <row r="9" spans="1:19" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="18" t="s">
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="18"/>
+      <c r="H9" s="7"/>
+      <c r="L9" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="S9" s="14"/>
     </row>
-    <row r="10" spans="1:19" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="15" t="s">
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="15"/>
+      <c r="H10" s="16"/>
+      <c r="L10" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="M10" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="S10" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
+  <mergeCells count="38">
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="R10:S10"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="L1:S1"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="M4:Q4"/>
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="B9:F9"/>
@@ -990,19 +1056,11 @@
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="L1:S1"/>
-    <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="R5:S5"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="REQUISITOS FUNCIONAIS">

</xml_diff>

<commit_message>
Doc: alteração do escopo, atualizando a tabela de requisitos
</commit_message>
<xml_diff>
--- a/documentacao/requisitos.xlsx
+++ b/documentacao/requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vieira\Desktop\Petsenai\documentacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B24BEC16-77CC-482E-A7E0-3F0E831381FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00DE25CA-2274-4708-9058-325D08934F5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{9C44EC18-CB13-4539-9BBD-338C7ACFB87E}"/>
   </bookViews>
@@ -327,6 +327,48 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -334,66 +376,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -730,316 +730,304 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="L1" s="21" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="L1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="21"/>
       <c r="L2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22" t="s">
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="22"/>
+      <c r="S2" s="14"/>
     </row>
     <row r="3" spans="1:19" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="16" t="s">
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="18"/>
       <c r="L3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="23" t="s">
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="23"/>
+      <c r="S3" s="17"/>
     </row>
     <row r="4" spans="1:19" ht="108" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="17" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="18"/>
+      <c r="H4" s="20"/>
       <c r="L4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="14" t="s">
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="S4" s="14"/>
+      <c r="S4" s="10"/>
     </row>
     <row r="5" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="17" t="s">
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
       <c r="L5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="M5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="22" t="s">
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="S5" s="22"/>
+      <c r="S5" s="14"/>
     </row>
     <row r="6" spans="1:19" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="17" t="s">
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="18"/>
+      <c r="H6" s="20"/>
       <c r="L6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="M6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="22" t="s">
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="S6" s="22"/>
+      <c r="S6" s="14"/>
     </row>
     <row r="7" spans="1:19" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="7" t="s">
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="21"/>
       <c r="L7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="M7" s="13" t="s">
+      <c r="M7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="14" t="s">
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="14"/>
+      <c r="S7" s="10"/>
     </row>
     <row r="8" spans="1:19" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="7" t="s">
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="21"/>
       <c r="L8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="M8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="24" t="s">
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="S8" s="24"/>
+      <c r="S8" s="13"/>
     </row>
     <row r="9" spans="1:19" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="7" t="s">
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="7"/>
-      <c r="L9" s="27" t="s">
+      <c r="H9" s="21"/>
+      <c r="L9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="M9" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="N9" s="15"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="14" t="s">
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="S9" s="14"/>
+      <c r="S9" s="10"/>
     </row>
     <row r="10" spans="1:19" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="16" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="16"/>
-      <c r="L10" s="27" t="s">
+      <c r="H10" s="18"/>
+      <c r="L10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="M10" s="13" t="s">
+      <c r="M10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="28" t="s">
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="S10" s="29"/>
+      <c r="S10" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="R9:S9"/>
-    <mergeCell ref="M10:Q10"/>
-    <mergeCell ref="R10:S10"/>
-    <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="R5:S5"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="R7:S7"/>
-    <mergeCell ref="L1:S1"/>
-    <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
     <mergeCell ref="M4:Q4"/>
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="B9:F9"/>
@@ -1056,11 +1044,23 @@
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="L1:S1"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="R10:S10"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="R8:S8"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="REQUISITOS FUNCIONAIS">
@@ -1068,5 +1068,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>